<commit_message>
Add Obramax, Cofema, Eletroleste and Smarfer to automations
- Add 4 new competitors: Obramax (home center atacado), Cofema
  Atacadista (CNPJ 69.194.454/0001-47), Eletroleste (Av. Aricanduva),
  and Smarfer to the competitor mapping (now 16 companies total)
- Add Obramax as price source for SUVINIL products including
  exclusive 20L packaging (Rende & Cobre, Toque Fosco, Glasu)
- Add Cofema, Eletroleste and Smarfer to scraping sources list
- Total: 15 products monitored across 32 price points

https://claude.ai/code/session_01D2AuCtbZF1Z8LTjB8AwAkC
</commit_message>
<xml_diff>
--- a/skills/ga-tintas-automation/output/concorrentes_ga_tintas.xlsx
+++ b/skills/ga-tintas-automation/output/concorrentes_ga_tintas.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Fontes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Concorrentes'!$A$4:$K$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Concorrentes'!$A$4:$K$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -513,7 +513,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mercado B2B de Tintas — São Paulo, SP | Gerado em: 20/03/2026 18:46</t>
+          <t>Mercado B2B de Tintas — São Paulo, SP | Gerado em: 20/03/2026 19:26</t>
         </is>
       </c>
     </row>
@@ -1258,8 +1258,236 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>OBRAMAX ATACADO S.A.</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Obramax</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Diversas lojas em São Paulo – SP e outras capitais</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>47.44-0/99 - Comércio varejista de materiais de construção em geral</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Grande</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Atacado e varejo de materiais de construção com ampla linha de tintas (Suvinil, Coral, etc.)</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Suvinil, Coral, e outras (75+ produtos Suvinil disponíveis)</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>CONCORRENTE DIRETO (Home center atacado)</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>obramax.com.br</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>COFEMA ATACADISTA LTDA</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Cofema Atacadista</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>69.194.454/0001-47</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Av. Aricanduva, 3241 – Vila Aricanduva, São Paulo – SP, CEP 03.527-000</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>46.72-9/00 - Comércio atacadista de ferragens e ferramentas</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Grande</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>R$ 18.860.000,00</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Atacadista de ferragens, ferramentas, tintas e materiais de construção — filiais em Sumaré, Bauru, Ribeirão Preto e Araçatuba</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Diversas marcas de tintas e materiais de construção</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>CONCORRENTE DIRETO (Atacadista materiais de construção)</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>cofema.com.br / Receita Federal</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>ELETROLESTE DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Eletroleste</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Av. Aricanduva, 5555 – São Paulo – SP</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>46.72-9/00 - Comércio atacadista de ferragens e ferramentas</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Atacadista de materiais hidráulicos, elétricos, ferramentas, tintas e máquinas</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Diversas marcas de tintas e materiais de construção</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>CONCORRENTE DIRETO (Atacadista regional)</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>eletroleste.com.br</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>SMARFER DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Smarfer</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>São Paulo – SP</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Distribuição de tintas e materiais de construção</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>CONCORRENTE DIRETO (A confirmar)</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Informação do cliente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:K16"/>
+  <autoFilter ref="A4:K20"/>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
@@ -1274,7 +1502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1355,7 +1583,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -1365,7 +1593,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -1469,17 +1697,34 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Obramax</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>CONCORRENTES INDIRETOS (overlap parcial)</t>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Cofema Atacadista</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>69.194.454/0001-47</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  → Tintas MC</t>
+          <t xml:space="preserve">  → Eletroleste</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1491,7 +1736,7 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  → Prema Tintas</t>
+          <t xml:space="preserve">  → Smarfer</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1500,37 +1745,68 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  → Tintas JD</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-    </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  → Tintas Irajá</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>60.910.023/0001-65</t>
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>CONCORRENTES INDIRETOS (overlap parcial)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  → Tintas MC</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Prema Tintas</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Tintas JD</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Tintas Irajá</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>60.910.023/0001-65</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">  → Martins Atacado</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>43.214.055/0001-07</t>
         </is>

</xml_diff>

<commit_message>
Fix Smarfer -> Ismafer (RA Martins Borges & Negócios LTDA)
Correct company name from "Smarfer" to "Ismafer" with proper data:
CNPJ 08.492.961/0004-15, capital social R$ 1M, comércio varejista
de ferragens e ferramentas em São Paulo.

https://claude.ai/code/session_01D2AuCtbZF1Z8LTjB8AwAkC
</commit_message>
<xml_diff>
--- a/skills/ga-tintas-automation/output/concorrentes_ga_tintas.xlsx
+++ b/skills/ga-tintas-automation/output/concorrentes_ga_tintas.xlsx
@@ -513,7 +513,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mercado B2B de Tintas — São Paulo, SP | Gerado em: 20/03/2026 19:26</t>
+          <t>Mercado B2B de Tintas — São Paulo, SP | Gerado em: 20/03/2026 20:00</t>
         </is>
       </c>
     </row>
@@ -1432,17 +1432,17 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>SMARFER DISTRIBUIDORA LTDA</t>
+          <t>RA MARTINS BORGES &amp; NEGÓCIOS LTDA</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Smarfer</t>
+          <t>Ismafer</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>08.492.961/0004-15</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -1452,37 +1452,37 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>47.44-0/01 - Comércio varejista de ferragens e ferramentas</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>R$ 1.000.000,00</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Distribuição de tintas e materiais de construção</t>
+          <t>Comércio varejista de ferragens, ferramentas, tintas e materiais de construção</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>Diversas marcas de ferramentas e tintas</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>CONCORRENTE DIRETO (A confirmar)</t>
+          <t>CONCORRENTE DIRETO (Varejo especializado)</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>Informação do cliente</t>
+          <t>Receita Federal / Econodata</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  → Smarfer</t>
+          <t xml:space="preserve">  → Ismafer</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>N/D</t>
+          <t>08.492.961/0004-15</t>
         </is>
       </c>
     </row>

</xml_diff>